<commit_message>
Auto update: 2025-12-10 02:38:27
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,43 +61,43 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2025-12-06</t>
+    <t>2025-12-10</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
+    <t>SK hynix</t>
+  </si>
+  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
-    <t>SK hynix</t>
+    <t>DB HiTek</t>
   </si>
   <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>005930.KS</t>
   </si>
   <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
+    <t>000660.KS</t>
+  </si>
+  <si>
     <t>058470.KS</t>
   </si>
   <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
-    <t>000660.KS</t>
+    <t>000990.KS</t>
   </si>
   <si>
     <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
   </si>
   <si>
     <t>Pattern</t>
@@ -528,25 +528,25 @@
         <v>108400</v>
       </c>
       <c r="E2">
-        <v>61.6</v>
+        <v>68.8</v>
       </c>
       <c r="F2">
-        <v>7.86</v>
+        <v>4.84</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H2">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="J2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="K2">
-        <v>54.7</v>
+        <v>58.8</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>65400</v>
+        <v>30400</v>
       </c>
       <c r="E3">
-        <v>61.7</v>
+        <v>53.1</v>
       </c>
       <c r="F3">
-        <v>-4.25</v>
+        <v>-2.88</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I3">
         <v>53</v>
       </c>
       <c r="J3">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K3">
-        <v>51.9</v>
+        <v>50.6</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>30300</v>
+        <v>566000</v>
       </c>
       <c r="E4">
-        <v>43.3</v>
+        <v>51.2</v>
       </c>
       <c r="F4">
-        <v>0.17</v>
+        <v>1.43</v>
       </c>
       <c r="G4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="I4">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J4">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="K4">
-        <v>50.7</v>
+        <v>48.8</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>544000</v>
+        <v>65200</v>
       </c>
       <c r="E5">
-        <v>33.8</v>
+        <v>66.7</v>
       </c>
       <c r="F5">
-        <v>2.64</v>
+        <v>-2.1</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I5">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="J5">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K5">
-        <v>48.1</v>
+        <v>47.8</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>61800</v>
+        <v>64900</v>
       </c>
       <c r="E6">
-        <v>38</v>
+        <v>47.4</v>
       </c>
       <c r="F6">
-        <v>0.82</v>
+        <v>-0.15</v>
       </c>
       <c r="G6">
         <v>20</v>
       </c>
       <c r="H6">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="I6">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="J6">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="K6">
-        <v>42.9</v>
+        <v>44.4</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>64800</v>
+        <v>61800</v>
       </c>
       <c r="E7">
-        <v>33.9</v>
+        <v>49</v>
       </c>
       <c r="F7">
-        <v>1.89</v>
+        <v>0.49</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="I7">
+        <v>30</v>
+      </c>
+      <c r="J7">
         <v>46</v>
       </c>
-      <c r="J7">
-        <v>63</v>
-      </c>
       <c r="K7">
-        <v>40.1</v>
+        <v>35.4</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>52.28493729186943</v>
+        <v>48.11568981226033</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2025-12-10 12:54:09
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -67,15 +67,15 @@
     <t>SamsungElec</t>
   </si>
   <si>
+    <t>SK hynix</t>
+  </si>
+  <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>SK hynix</t>
-  </si>
-  <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
     <t>DB HiTek</t>
   </si>
   <si>
@@ -85,13 +85,13 @@
     <t>005930.KS</t>
   </si>
   <si>
+    <t>000660.KS</t>
+  </si>
+  <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
     <t>403870.KS</t>
-  </si>
-  <si>
-    <t>000660.KS</t>
-  </si>
-  <si>
-    <t>058470.KS</t>
   </si>
   <si>
     <t>000990.KS</t>
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>108400</v>
+        <v>108600</v>
       </c>
       <c r="E2">
-        <v>68.8</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="F2">
-        <v>4.84</v>
+        <v>3.92</v>
       </c>
       <c r="G2">
         <v>60</v>
       </c>
       <c r="H2">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I2">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="K2">
-        <v>58.8</v>
+        <v>59.9</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>30400</v>
+        <v>587500</v>
       </c>
       <c r="E3">
-        <v>53.1</v>
+        <v>54.2</v>
       </c>
       <c r="F3">
-        <v>-2.88</v>
+        <v>6.43</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I3">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="J3">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K3">
-        <v>50.6</v>
+        <v>56.9</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,16 +619,16 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>566000</v>
+        <v>65300</v>
       </c>
       <c r="E4">
-        <v>51.2</v>
+        <v>69</v>
       </c>
       <c r="F4">
-        <v>1.43</v>
+        <v>-0.46</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H4">
         <v>66</v>
@@ -637,10 +637,10 @@
         <v>56</v>
       </c>
       <c r="J4">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K4">
-        <v>48.8</v>
+        <v>51.3</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>65200</v>
+        <v>30100</v>
       </c>
       <c r="E5">
-        <v>66.7</v>
+        <v>57</v>
       </c>
       <c r="F5">
-        <v>-2.1</v>
+        <v>-3.68</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I5">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="J5">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="K5">
-        <v>47.8</v>
+        <v>49.9</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>64900</v>
+        <v>66000</v>
       </c>
       <c r="E6">
-        <v>47.4</v>
+        <v>48.7</v>
       </c>
       <c r="F6">
-        <v>-0.15</v>
+        <v>0.61</v>
       </c>
       <c r="G6">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H6">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J6">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="K6">
-        <v>44.4</v>
+        <v>46.1</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -763,25 +763,25 @@
         <v>61800</v>
       </c>
       <c r="E7">
-        <v>49</v>
+        <v>52.6</v>
       </c>
       <c r="F7">
-        <v>0.49</v>
+        <v>0.16</v>
       </c>
       <c r="G7">
         <v>30</v>
       </c>
       <c r="H7">
+        <v>40</v>
+      </c>
+      <c r="I7">
         <v>43</v>
       </c>
-      <c r="I7">
-        <v>30</v>
-      </c>
       <c r="J7">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="K7">
-        <v>35.4</v>
+        <v>40.1</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>48.11568981226033</v>
+        <v>46.17217538625081</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2025-12-15 01:10:22
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -61,7 +61,7 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2025-12-10</t>
+    <t>2025-12-15</t>
   </si>
   <si>
     <t>SamsungElec</t>
@@ -70,37 +70,40 @@
     <t>SK hynix</t>
   </si>
   <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
     <t>005930.KS</t>
   </si>
   <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>058470.KS</t>
   </si>
   <si>
     <t>403870.KS</t>
   </si>
   <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
+  </si>
+  <si>
+    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -525,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>108600</v>
+        <v>108900</v>
       </c>
       <c r="E2">
-        <v>64.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="F2">
-        <v>3.92</v>
+        <v>0.46</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H2">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I2">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="J2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="K2">
-        <v>59.9</v>
+        <v>62.4</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -572,40 +575,40 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>587500</v>
+        <v>571000</v>
       </c>
       <c r="E3">
-        <v>54.2</v>
+        <v>64.3</v>
       </c>
       <c r="F3">
-        <v>6.43</v>
+        <v>4.96</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I3">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="J3">
         <v>66</v>
       </c>
       <c r="K3">
-        <v>56.9</v>
+        <v>55.6</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,40 +622,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>65300</v>
+        <v>67600</v>
       </c>
       <c r="E4">
-        <v>69</v>
+        <v>79.3</v>
       </c>
       <c r="F4">
-        <v>-0.46</v>
+        <v>4.32</v>
       </c>
       <c r="G4">
         <v>50</v>
       </c>
       <c r="H4">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="I4">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J4">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="K4">
-        <v>51.3</v>
+        <v>53.2</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -666,40 +669,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>30100</v>
+        <v>62400</v>
       </c>
       <c r="E5">
-        <v>57</v>
+        <v>65.7</v>
       </c>
       <c r="F5">
-        <v>-3.68</v>
+        <v>0.97</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J5">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="K5">
-        <v>49.9</v>
+        <v>49.2</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N5">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -713,40 +716,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>66000</v>
+        <v>63600</v>
       </c>
       <c r="E6">
-        <v>48.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F6">
-        <v>0.61</v>
+        <v>-2.75</v>
       </c>
       <c r="G6">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="I6">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="J6">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K6">
-        <v>46.1</v>
+        <v>47.4</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,40 +763,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>61800</v>
+        <v>29450</v>
       </c>
       <c r="E7">
-        <v>52.6</v>
+        <v>62.1</v>
       </c>
       <c r="F7">
-        <v>0.16</v>
+        <v>-2.81</v>
       </c>
       <c r="G7">
         <v>30</v>
       </c>
       <c r="H7">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="I7">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="J7">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="K7">
-        <v>40.1</v>
+        <v>44.4</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7">
-        <v>46.17217538625081</v>
+        <v>47.37006702605126</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2025-12-29 23:08:35
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>날짜</t>
   </si>
@@ -61,49 +61,46 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2025-12-15</t>
+    <t>2025-12-29</t>
+  </si>
+  <si>
+    <t>SK hynix</t>
+  </si>
+  <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
-    <t>SK hynix</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
+    <t>000660.KS</t>
+  </si>
+  <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
+    <t>403870.KS</t>
   </si>
   <si>
     <t>005930.KS</t>
   </si>
   <si>
-    <t>000660.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
     <t>240810.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
   </si>
   <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
-  </si>
-  <si>
-    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -528,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>108900</v>
+        <v>640000</v>
       </c>
       <c r="E2">
-        <v>77</v>
+        <v>64.3</v>
       </c>
       <c r="F2">
-        <v>0.46</v>
+        <v>17</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="I2">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="J2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="K2">
-        <v>62.4</v>
+        <v>55.8</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,10 +555,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>47.37006702605126</v>
+        <v>51.940834218365</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -575,40 +572,40 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>571000</v>
+        <v>67100</v>
       </c>
       <c r="E3">
-        <v>64.3</v>
+        <v>53.2</v>
       </c>
       <c r="F3">
-        <v>4.96</v>
+        <v>2.76</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H3">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I3">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="J3">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="K3">
-        <v>55.6</v>
+        <v>54.8</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3">
+        <v>51.940834218365</v>
+      </c>
+      <c r="O3" t="s">
         <v>30</v>
-      </c>
-      <c r="N3">
-        <v>47.37006702605126</v>
-      </c>
-      <c r="O3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -622,40 +619,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>67600</v>
+        <v>30950</v>
       </c>
       <c r="E4">
-        <v>79.3</v>
+        <v>54.4</v>
       </c>
       <c r="F4">
-        <v>4.32</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="G4">
+        <v>60</v>
+      </c>
+      <c r="H4">
+        <v>56</v>
+      </c>
+      <c r="I4">
         <v>50</v>
       </c>
-      <c r="H4">
-        <v>46</v>
-      </c>
-      <c r="I4">
-        <v>60</v>
-      </c>
       <c r="J4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="K4">
-        <v>53.2</v>
+        <v>53.6</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4">
+        <v>51.940834218365</v>
+      </c>
+      <c r="O4" t="s">
         <v>30</v>
-      </c>
-      <c r="N4">
-        <v>47.37006702605126</v>
-      </c>
-      <c r="O4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -669,40 +666,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>62400</v>
+        <v>119500</v>
       </c>
       <c r="E5">
-        <v>65.7</v>
+        <v>66.3</v>
       </c>
       <c r="F5">
-        <v>0.97</v>
+        <v>12.42</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="H5">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="I5">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J5">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="K5">
-        <v>49.2</v>
+        <v>53</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5">
+        <v>51.940834218365</v>
+      </c>
+      <c r="O5" t="s">
         <v>30</v>
-      </c>
-      <c r="N5">
-        <v>47.37006702605126</v>
-      </c>
-      <c r="O5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -716,40 +713,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>63600</v>
+        <v>67900</v>
       </c>
       <c r="E6">
-        <v>68.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="F6">
-        <v>-2.75</v>
+        <v>18.91</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H6">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I6">
         <v>53</v>
       </c>
       <c r="J6">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="K6">
-        <v>47.4</v>
+        <v>51.8</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6">
+        <v>51.940834218365</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
-      </c>
-      <c r="N6">
-        <v>47.37006702605126</v>
-      </c>
-      <c r="O6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -763,40 +760,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>29450</v>
+        <v>61100</v>
       </c>
       <c r="E7">
-        <v>62.1</v>
+        <v>32.2</v>
       </c>
       <c r="F7">
-        <v>-2.81</v>
+        <v>1.83</v>
       </c>
       <c r="G7">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H7">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="I7">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J7">
         <v>60</v>
       </c>
       <c r="K7">
-        <v>44.4</v>
+        <v>40</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7">
+        <v>51.940834218365</v>
+      </c>
+      <c r="O7" t="s">
         <v>30</v>
-      </c>
-      <c r="N7">
-        <v>47.37006702605126</v>
-      </c>
-      <c r="O7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-01-05 00:38:42
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,43 +61,43 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2025-12-29</t>
+    <t>2026-01-05</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
     <t>DB HiTek</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
     <t>000990.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
-    <t>005930.KS</t>
-  </si>
-  <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>058470.KS</t>
   </si>
   <si>
     <t>Pattern</t>
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>640000</v>
+        <v>677000</v>
       </c>
       <c r="E2">
-        <v>64.3</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F2">
-        <v>17</v>
+        <v>15.92</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I2">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="J2">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="K2">
-        <v>55.8</v>
+        <v>49.9</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>67100</v>
+        <v>80000</v>
       </c>
       <c r="E3">
-        <v>53.2</v>
+        <v>69</v>
       </c>
       <c r="F3">
-        <v>2.76</v>
+        <v>27.39</v>
       </c>
       <c r="G3">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H3">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I3">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="J3">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="K3">
-        <v>54.8</v>
+        <v>49.9</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>30950</v>
+        <v>34450</v>
       </c>
       <c r="E4">
-        <v>54.4</v>
+        <v>74</v>
       </c>
       <c r="F4">
-        <v>8.220000000000001</v>
+        <v>13.32</v>
       </c>
       <c r="G4">
+        <v>40</v>
+      </c>
+      <c r="H4">
         <v>60</v>
       </c>
-      <c r="H4">
-        <v>56</v>
-      </c>
       <c r="I4">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J4">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K4">
-        <v>53.6</v>
+        <v>48.5</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>119500</v>
+        <v>64900</v>
       </c>
       <c r="E5">
-        <v>66.3</v>
+        <v>53.5</v>
       </c>
       <c r="F5">
-        <v>12.42</v>
+        <v>5.7</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I5">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J5">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="K5">
-        <v>53</v>
+        <v>48.5</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>67900</v>
+        <v>128500</v>
       </c>
       <c r="E6">
-        <v>61</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="F6">
-        <v>18.91</v>
+        <v>15.25</v>
       </c>
       <c r="G6">
+        <v>40</v>
+      </c>
+      <c r="H6">
         <v>50</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>56</v>
       </c>
-      <c r="I6">
-        <v>53</v>
-      </c>
       <c r="J6">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K6">
-        <v>51.8</v>
+        <v>46.9</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,16 +760,16 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>61100</v>
+        <v>73700</v>
       </c>
       <c r="E7">
-        <v>32.2</v>
+        <v>69</v>
       </c>
       <c r="F7">
-        <v>1.83</v>
+        <v>6.2</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H7">
         <v>46</v>
@@ -778,10 +778,10 @@
         <v>46</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="K7">
-        <v>40</v>
+        <v>45.9</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>51.940834218365</v>
+        <v>41.50472307187444</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-07 10:56:12
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,43 +61,43 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-05</t>
+    <t>2026-01-07</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
     <t>240810.KS</t>
   </si>
   <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
     <t>403870.KS</t>
-  </si>
-  <si>
-    <t>058470.KS</t>
-  </si>
-  <si>
-    <t>005930.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
   </si>
   <si>
     <t>Pattern</t>
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>677000</v>
+        <v>754000</v>
       </c>
       <c r="E2">
-        <v>69.90000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="F2">
-        <v>15.92</v>
+        <v>17.81</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="I2">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="J2">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="K2">
-        <v>49.9</v>
+        <v>57.5</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>80000</v>
+        <v>142300</v>
       </c>
       <c r="E3">
-        <v>69</v>
+        <v>91.2</v>
       </c>
       <c r="F3">
-        <v>27.39</v>
+        <v>19.08</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I3">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="J3">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="K3">
-        <v>49.9</v>
+        <v>54.7</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>34450</v>
+        <v>66300</v>
       </c>
       <c r="E4">
-        <v>74</v>
+        <v>58.7</v>
       </c>
       <c r="F4">
-        <v>13.32</v>
+        <v>8.51</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I4">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="J4">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="K4">
-        <v>48.5</v>
+        <v>53.9</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>64900</v>
+        <v>80400</v>
       </c>
       <c r="E5">
-        <v>53.5</v>
+        <v>70</v>
       </c>
       <c r="F5">
-        <v>5.7</v>
+        <v>18.41</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J5">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K5">
-        <v>48.5</v>
+        <v>53.7</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>128500</v>
+        <v>74500</v>
       </c>
       <c r="E6">
-        <v>76.90000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F6">
-        <v>15.25</v>
+        <v>11.03</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I6">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J6">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="K6">
-        <v>46.9</v>
+        <v>49.7</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>73700</v>
+        <v>39150</v>
       </c>
       <c r="E7">
-        <v>69</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F7">
-        <v>6.2</v>
+        <v>26.49</v>
       </c>
       <c r="G7">
+        <v>40</v>
+      </c>
+      <c r="H7">
         <v>50</v>
       </c>
-      <c r="H7">
-        <v>46</v>
-      </c>
       <c r="I7">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J7">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K7">
-        <v>45.9</v>
+        <v>45.5</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>41.50472307187444</v>
+        <v>45.04298008974126</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-07 14:23:17
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>754000</v>
+        <v>735000</v>
       </c>
       <c r="E2">
-        <v>88.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="F2">
-        <v>17.81</v>
+        <v>14.84</v>
       </c>
       <c r="G2">
         <v>40</v>
       </c>
       <c r="H2">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I2">
         <v>80</v>
       </c>
       <c r="J2">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="K2">
-        <v>57.5</v>
+        <v>57.6</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,13 +572,13 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>142300</v>
+        <v>138700</v>
       </c>
       <c r="E3">
-        <v>91.2</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="F3">
-        <v>19.08</v>
+        <v>16.07</v>
       </c>
       <c r="G3">
         <v>40</v>
@@ -593,7 +593,7 @@
         <v>83</v>
       </c>
       <c r="K3">
-        <v>54.7</v>
+        <v>54.8</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -640,7 +640,7 @@
         <v>76</v>
       </c>
       <c r="K4">
-        <v>53.9</v>
+        <v>54</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -687,7 +687,7 @@
         <v>70</v>
       </c>
       <c r="K5">
-        <v>53.7</v>
+        <v>53.8</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,13 +713,13 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>74500</v>
+        <v>73400</v>
       </c>
       <c r="E6">
-        <v>74.90000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F6">
-        <v>11.03</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="G6">
         <v>50</v>
@@ -734,7 +734,7 @@
         <v>63</v>
       </c>
       <c r="K6">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -781,7 +781,7 @@
         <v>60</v>
       </c>
       <c r="K7">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>45.04298008974126</v>
+        <v>45.26531441048893</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-08 15:59:52
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,40 +61,40 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-07</t>
+    <t>2026-01-08</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
     <t>SamsungElec</t>
   </si>
   <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
     <t>005930.KS</t>
   </si>
   <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>058470.KS</t>
-  </si>
-  <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
   </si>
   <si>
     <t>403870.KS</t>
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>735000</v>
+        <v>756000</v>
       </c>
       <c r="E2">
-        <v>87.90000000000001</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F2">
-        <v>14.84</v>
+        <v>16.13</v>
       </c>
       <c r="G2">
         <v>40</v>
       </c>
       <c r="H2">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J2">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="K2">
-        <v>57.6</v>
+        <v>54.3</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>138700</v>
+        <v>71700</v>
       </c>
       <c r="E3">
-        <v>90.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="F3">
-        <v>16.07</v>
+        <v>6.07</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="I3">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="J3">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K3">
-        <v>54.8</v>
+        <v>53.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>66300</v>
+        <v>138800</v>
       </c>
       <c r="E4">
-        <v>58.7</v>
+        <v>90.5</v>
       </c>
       <c r="F4">
-        <v>8.51</v>
+        <v>15.76</v>
       </c>
       <c r="G4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H4">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="I4">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J4">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="K4">
-        <v>54</v>
+        <v>53.3</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>80400</v>
+        <v>78900</v>
       </c>
       <c r="E5">
-        <v>70</v>
+        <v>70.8</v>
       </c>
       <c r="F5">
-        <v>18.41</v>
+        <v>21.57</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="H5">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I5">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J5">
         <v>70</v>
       </c>
       <c r="K5">
-        <v>53.8</v>
+        <v>52.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>73400</v>
+        <v>64200</v>
       </c>
       <c r="E6">
-        <v>70.59999999999999</v>
+        <v>58.3</v>
       </c>
       <c r="F6">
-        <v>9.390000000000001</v>
+        <v>5.42</v>
       </c>
       <c r="G6">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H6">
         <v>56</v>
       </c>
       <c r="I6">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J6">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="K6">
-        <v>49.8</v>
+        <v>51.1</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>39150</v>
+        <v>33200</v>
       </c>
       <c r="E7">
-        <v>83.40000000000001</v>
+        <v>61</v>
       </c>
       <c r="F7">
-        <v>26.49</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I7">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="K7">
-        <v>45.6</v>
+        <v>49.3</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>45.26531441048893</v>
+        <v>43.60821037092016</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-11 19:20:10
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -61,46 +61,49 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-08</t>
+    <t>2026-01-11</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>DB HiTek</t>
   </si>
   <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>000990.KS</t>
   </si>
   <si>
-    <t>005930.KS</t>
-  </si>
-  <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>058470.KS</t>
-  </si>
-  <si>
     <t>403870.KS</t>
   </si>
   <si>
     <t>Pattern</t>
+  </si>
+  <si>
+    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -525,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>756000</v>
+        <v>744000</v>
       </c>
       <c r="E2">
-        <v>97.90000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="F2">
-        <v>16.13</v>
+        <v>9.9</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H2">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="I2">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J2">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K2">
-        <v>54.3</v>
+        <v>60.5</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -572,40 +575,40 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>71700</v>
+        <v>139000</v>
       </c>
       <c r="E3">
-        <v>65.2</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F3">
-        <v>6.07</v>
+        <v>8.17</v>
       </c>
       <c r="G3">
+        <v>50</v>
+      </c>
+      <c r="H3">
         <v>60</v>
       </c>
-      <c r="H3">
-        <v>53</v>
-      </c>
       <c r="I3">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="J3">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="K3">
-        <v>53.5</v>
+        <v>56.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,40 +622,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>138800</v>
+        <v>62700</v>
       </c>
       <c r="E4">
-        <v>90.5</v>
+        <v>58.6</v>
       </c>
       <c r="F4">
-        <v>15.76</v>
+        <v>-3.39</v>
       </c>
       <c r="G4">
         <v>50</v>
       </c>
       <c r="H4">
+        <v>56</v>
+      </c>
+      <c r="I4">
+        <v>66</v>
+      </c>
+      <c r="J4">
         <v>63</v>
       </c>
-      <c r="I4">
-        <v>63</v>
-      </c>
-      <c r="J4">
-        <v>86</v>
-      </c>
       <c r="K4">
-        <v>53.3</v>
+        <v>56.5</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -666,19 +669,19 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>78900</v>
+        <v>75000</v>
       </c>
       <c r="E5">
-        <v>70.8</v>
+        <v>62.5</v>
       </c>
       <c r="F5">
-        <v>21.57</v>
+        <v>-6.25</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="H5">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="I5">
         <v>60</v>
@@ -687,19 +690,19 @@
         <v>70</v>
       </c>
       <c r="K5">
-        <v>52.1</v>
+        <v>54.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N5">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -713,40 +716,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>64200</v>
+        <v>71900</v>
       </c>
       <c r="E6">
-        <v>58.3</v>
+        <v>65.2</v>
       </c>
       <c r="F6">
-        <v>5.42</v>
+        <v>-2.44</v>
       </c>
       <c r="G6">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H6">
         <v>56</v>
       </c>
       <c r="I6">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J6">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K6">
-        <v>51.1</v>
+        <v>52.5</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,40 +763,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>33200</v>
+        <v>33100</v>
       </c>
       <c r="E7">
-        <v>61</v>
+        <v>59.2</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>-3.92</v>
       </c>
       <c r="G7">
         <v>50</v>
       </c>
       <c r="H7">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I7">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J7">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="K7">
-        <v>49.3</v>
+        <v>50.1</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7">
-        <v>43.60821037092016</v>
+        <v>50.40292622392195</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-01-12 10:56:40
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,7 +61,7 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-11</t>
+    <t>2026-01-12</t>
   </si>
   <si>
     <t>SK hynix</t>
@@ -76,12 +76,12 @@
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
     <t>DB HiTek</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
     <t>000660.KS</t>
   </si>
   <si>
@@ -94,10 +94,10 @@
     <t>240810.KS</t>
   </si>
   <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
     <t>000990.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
   </si>
   <si>
     <t>Pattern</t>
@@ -528,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>744000</v>
+        <v>758000</v>
       </c>
       <c r="E2">
-        <v>92.5</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F2">
-        <v>9.9</v>
+        <v>8.91</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="I2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="K2">
-        <v>60.5</v>
+        <v>62.1</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,13 +575,13 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>139000</v>
+        <v>140300</v>
       </c>
       <c r="E3">
-        <v>89.40000000000001</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="F3">
-        <v>8.17</v>
+        <v>1.59</v>
       </c>
       <c r="G3">
         <v>50</v>
@@ -590,22 +590,22 @@
         <v>60</v>
       </c>
       <c r="I3">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J3">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="K3">
-        <v>56.5</v>
+        <v>60.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N3">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -652,7 +652,7 @@
         <v>30</v>
       </c>
       <c r="N4">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -681,16 +681,16 @@
         <v>50</v>
       </c>
       <c r="H5">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="J5">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="K5">
-        <v>54.1</v>
+        <v>56.5</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>30</v>
       </c>
       <c r="N5">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -716,28 +716,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>71900</v>
+        <v>33100</v>
       </c>
       <c r="E6">
-        <v>65.2</v>
+        <v>59.2</v>
       </c>
       <c r="F6">
-        <v>-2.44</v>
+        <v>-3.92</v>
       </c>
       <c r="G6">
         <v>50</v>
       </c>
       <c r="H6">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I6">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="J6">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="K6">
-        <v>52.5</v>
+        <v>50.1</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
       <c r="N6">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,28 +763,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>33100</v>
+        <v>74400</v>
       </c>
       <c r="E7">
-        <v>59.2</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F7">
-        <v>-3.92</v>
+        <v>-1.06</v>
       </c>
       <c r="G7">
+        <v>40</v>
+      </c>
+      <c r="H7">
         <v>50</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>53</v>
       </c>
-      <c r="I7">
-        <v>50</v>
-      </c>
       <c r="J7">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="K7">
-        <v>50.1</v>
+        <v>48.3</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -793,7 +793,7 @@
         <v>30</v>
       </c>
       <c r="N7">
-        <v>50.40292622392195</v>
+        <v>50.43822221555986</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-12 16:23:22
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -64,12 +64,12 @@
     <t>2026-01-12</t>
   </si>
   <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
     <t>SK hynix</t>
   </si>
   <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
@@ -82,10 +82,10 @@
     <t>DB HiTek</t>
   </si>
   <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
     <t>000660.KS</t>
-  </si>
-  <si>
-    <t>005930.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
@@ -528,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>758000</v>
+        <v>138800</v>
       </c>
       <c r="E2">
-        <v>92.90000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F2">
-        <v>8.91</v>
+        <v>0.51</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="J2">
         <v>90</v>
       </c>
       <c r="K2">
-        <v>62.1</v>
+        <v>60.6</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,28 +575,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>140300</v>
+        <v>749000</v>
       </c>
       <c r="E3">
-        <v>90.40000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="F3">
-        <v>1.59</v>
+        <v>7.61</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="I3">
         <v>76</v>
       </c>
       <c r="J3">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="K3">
-        <v>60.5</v>
+        <v>60.6</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,7 +605,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -643,7 +643,7 @@
         <v>63</v>
       </c>
       <c r="K4">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -652,7 +652,7 @@
         <v>30</v>
       </c>
       <c r="N4">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -690,7 +690,7 @@
         <v>76</v>
       </c>
       <c r="K5">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>30</v>
       </c>
       <c r="N5">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -737,7 +737,7 @@
         <v>43</v>
       </c>
       <c r="K6">
-        <v>50.1</v>
+        <v>50.2</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
       <c r="N6">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,13 +763,13 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>74400</v>
+        <v>74000</v>
       </c>
       <c r="E7">
-        <v>73.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F7">
-        <v>-1.06</v>
+        <v>-1.6</v>
       </c>
       <c r="G7">
         <v>40</v>
@@ -784,7 +784,7 @@
         <v>60</v>
       </c>
       <c r="K7">
-        <v>48.3</v>
+        <v>48.4</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -793,7 +793,7 @@
         <v>30</v>
       </c>
       <c r="N7">
-        <v>50.43822221555986</v>
+        <v>50.56766494832259</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-13 13:54:43
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>날짜</t>
   </si>
@@ -61,49 +61,46 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-12</t>
+    <t>2026-01-13</t>
+  </si>
+  <si>
+    <t>SK hynix</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
-    <t>SK hynix</t>
+    <t>DB HiTek</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
+    <t>000660.KS</t>
   </si>
   <si>
     <t>005930.KS</t>
   </si>
   <si>
-    <t>000660.KS</t>
+    <t>000990.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
   </si>
   <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
     <t>240810.KS</t>
   </si>
   <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
-  </si>
-  <si>
-    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -528,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>138800</v>
+        <v>726000</v>
       </c>
       <c r="E2">
-        <v>89.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="F2">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="I2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="J2">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="K2">
-        <v>60.6</v>
+        <v>58.4</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,10 +555,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>50.56766494832259</v>
+        <v>47.98314273412904</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -575,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>749000</v>
+        <v>137100</v>
       </c>
       <c r="E3">
-        <v>92.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="F3">
-        <v>7.61</v>
+        <v>-1.3</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I3">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J3">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="K3">
-        <v>60.6</v>
+        <v>55.6</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,10 +602,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>50.56766494832259</v>
+        <v>47.98314273412904</v>
       </c>
       <c r="O3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -622,40 +619,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>62700</v>
+        <v>76200</v>
       </c>
       <c r="E4">
-        <v>58.6</v>
+        <v>74.2</v>
       </c>
       <c r="F4">
-        <v>-3.39</v>
+        <v>1.33</v>
       </c>
       <c r="G4">
         <v>50</v>
       </c>
       <c r="H4">
+        <v>43</v>
+      </c>
+      <c r="I4">
         <v>56</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>66</v>
       </c>
-      <c r="J4">
-        <v>63</v>
-      </c>
       <c r="K4">
-        <v>56.6</v>
+        <v>51.8</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4">
+        <v>47.98314273412904</v>
+      </c>
+      <c r="O4" t="s">
         <v>30</v>
-      </c>
-      <c r="N4">
-        <v>50.56766494832259</v>
-      </c>
-      <c r="O4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -669,40 +666,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>75000</v>
+        <v>62900</v>
       </c>
       <c r="E5">
-        <v>62.5</v>
+        <v>60.4</v>
       </c>
       <c r="F5">
-        <v>-6.25</v>
+        <v>-3.23</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="H5">
+        <v>50</v>
+      </c>
+      <c r="I5">
         <v>53</v>
       </c>
-      <c r="I5">
-        <v>66</v>
-      </c>
       <c r="J5">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="K5">
-        <v>56.6</v>
+        <v>50.6</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5">
+        <v>47.98314273412904</v>
+      </c>
+      <c r="O5" t="s">
         <v>30</v>
-      </c>
-      <c r="N5">
-        <v>50.56766494832259</v>
-      </c>
-      <c r="O5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -716,40 +713,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>33100</v>
+        <v>33600</v>
       </c>
       <c r="E6">
-        <v>59.2</v>
+        <v>62.4</v>
       </c>
       <c r="F6">
-        <v>-3.92</v>
+        <v>-4</v>
       </c>
       <c r="G6">
         <v>50</v>
       </c>
       <c r="H6">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>50</v>
       </c>
       <c r="J6">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="K6">
-        <v>50.2</v>
+        <v>49.4</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6">
+        <v>47.98314273412904</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
-      </c>
-      <c r="N6">
-        <v>50.56766494832259</v>
-      </c>
-      <c r="O6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -763,40 +760,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>74000</v>
+        <v>73300</v>
       </c>
       <c r="E7">
-        <v>73.09999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="F7">
-        <v>-1.6</v>
+        <v>-6.98</v>
       </c>
       <c r="G7">
         <v>40</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I7">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="K7">
-        <v>48.4</v>
+        <v>44.8</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7">
+        <v>47.98314273412904</v>
+      </c>
+      <c r="O7" t="s">
         <v>30</v>
-      </c>
-      <c r="N7">
-        <v>50.56766494832259</v>
-      </c>
-      <c r="O7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-01-14 16:48:58
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,43 +61,43 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-13</t>
+    <t>2026-01-14</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
     <t>SamsungElec</t>
   </si>
   <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>DB HiTek</t>
   </si>
   <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
     <t>005930.KS</t>
   </si>
   <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>000990.KS</t>
-  </si>
-  <si>
-    <t>058470.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
-    <t>240810.KS</t>
   </si>
   <si>
     <t>Pattern</t>
@@ -525,10 +525,10 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>726000</v>
+        <v>742000</v>
       </c>
       <c r="E2">
-        <v>85.90000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -537,16 +537,16 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="K2">
-        <v>58.4</v>
+        <v>58.1</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>137100</v>
+        <v>63600</v>
       </c>
       <c r="E3">
-        <v>88.7</v>
+        <v>64.5</v>
       </c>
       <c r="F3">
-        <v>-1.3</v>
+        <v>-4.07</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H3">
+        <v>63</v>
+      </c>
+      <c r="I3">
+        <v>63</v>
+      </c>
+      <c r="J3">
         <v>70</v>
       </c>
-      <c r="I3">
-        <v>73</v>
-      </c>
-      <c r="J3">
-        <v>83</v>
-      </c>
       <c r="K3">
-        <v>55.6</v>
+        <v>53.1</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>76200</v>
+        <v>140300</v>
       </c>
       <c r="E4">
-        <v>74.2</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F4">
-        <v>1.33</v>
+        <v>-0.5</v>
       </c>
       <c r="G4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="I4">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="J4">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="K4">
-        <v>51.8</v>
+        <v>52.9</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,13 +666,13 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>62900</v>
+        <v>33450</v>
       </c>
       <c r="E5">
-        <v>60.4</v>
+        <v>61.7</v>
       </c>
       <c r="F5">
-        <v>-3.23</v>
+        <v>-14.56</v>
       </c>
       <c r="G5">
         <v>50</v>
@@ -681,13 +681,13 @@
         <v>50</v>
       </c>
       <c r="I5">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J5">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K5">
-        <v>50.6</v>
+        <v>47.9</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>33600</v>
+        <v>75900</v>
       </c>
       <c r="E6">
-        <v>62.4</v>
+        <v>72.2</v>
       </c>
       <c r="F6">
-        <v>-4</v>
+        <v>-5.6</v>
       </c>
       <c r="G6">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I6">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J6">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="K6">
-        <v>49.4</v>
+        <v>47.3</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>73300</v>
+        <v>81900</v>
       </c>
       <c r="E7">
-        <v>70.7</v>
+        <v>77</v>
       </c>
       <c r="F7">
-        <v>-6.98</v>
+        <v>10.38</v>
       </c>
       <c r="G7">
         <v>40</v>
       </c>
       <c r="H7">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="I7">
         <v>46</v>
       </c>
       <c r="J7">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="K7">
-        <v>44.8</v>
+        <v>43.3</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>47.98314273412904</v>
+        <v>43.1153238131143</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-01-17 15:48:26
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -61,46 +61,49 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-14</t>
+    <t>2026-01-17</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
     <t>058470.KS</t>
   </si>
   <si>
-    <t>005930.KS</t>
-  </si>
-  <si>
     <t>403870.KS</t>
   </si>
   <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
+  </si>
+  <si>
+    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -525,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>742000</v>
+        <v>756000</v>
       </c>
       <c r="E2">
-        <v>88.90000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1.61</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H2">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I2">
         <v>83</v>
       </c>
       <c r="J2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K2">
-        <v>58.1</v>
+        <v>60.3</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -572,40 +575,40 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>63600</v>
+        <v>76700</v>
       </c>
       <c r="E3">
-        <v>64.5</v>
+        <v>67.3</v>
       </c>
       <c r="F3">
-        <v>-4.07</v>
+        <v>2.27</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H3">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I3">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J3">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="K3">
-        <v>53.1</v>
+        <v>54.1</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,40 +622,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>140300</v>
+        <v>148900</v>
       </c>
       <c r="E4">
-        <v>89.40000000000001</v>
+        <v>92</v>
       </c>
       <c r="F4">
-        <v>-0.5</v>
+        <v>7.12</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H4">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I4">
+        <v>56</v>
+      </c>
+      <c r="J4">
         <v>70</v>
       </c>
-      <c r="J4">
-        <v>76</v>
-      </c>
       <c r="K4">
-        <v>52.9</v>
+        <v>49.5</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -666,40 +669,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>33450</v>
+        <v>85200</v>
       </c>
       <c r="E5">
-        <v>61.7</v>
+        <v>81.5</v>
       </c>
       <c r="F5">
-        <v>-14.56</v>
+        <v>18.5</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I5">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J5">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="K5">
-        <v>47.9</v>
+        <v>48.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N5">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -713,25 +716,25 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>75900</v>
+        <v>64700</v>
       </c>
       <c r="E6">
-        <v>72.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F6">
-        <v>-5.6</v>
+        <v>3.19</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H6">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I6">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="J6">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="K6">
         <v>47.3</v>
@@ -740,13 +743,13 @@
         <v>28</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,40 +763,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>81900</v>
+        <v>35750</v>
       </c>
       <c r="E7">
-        <v>77</v>
+        <v>63.9</v>
       </c>
       <c r="F7">
-        <v>10.38</v>
+        <v>8.01</v>
       </c>
       <c r="G7">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H7">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I7">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="J7">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K7">
-        <v>43.3</v>
+        <v>44.5</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7">
-        <v>43.1153238131143</v>
+        <v>40.49436870247035</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-01-19 15:55:40
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>날짜</t>
   </si>
@@ -61,7 +61,7 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-17</t>
+    <t>2026-01-19</t>
   </si>
   <si>
     <t>SK hynix</t>
@@ -101,9 +101,6 @@
   </si>
   <si>
     <t>Pattern</t>
-  </si>
-  <si>
-    <t>📈 매수 관찰 구간입니다.</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
@@ -528,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>756000</v>
+        <v>764000</v>
       </c>
       <c r="E2">
-        <v>89.3</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="F2">
-        <v>1.61</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
+        <v>80</v>
+      </c>
+      <c r="I2">
         <v>76</v>
       </c>
-      <c r="I2">
-        <v>83</v>
-      </c>
       <c r="J2">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="K2">
-        <v>60.3</v>
+        <v>57.5</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,10 +555,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>40.49436870247035</v>
+        <v>40.44495449250464</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -587,28 +584,28 @@
         <v>60</v>
       </c>
       <c r="H3">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I3">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="J3">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="K3">
-        <v>54.1</v>
+        <v>56.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3">
+        <v>40.44495449250464</v>
+      </c>
+      <c r="O3" t="s">
         <v>30</v>
-      </c>
-      <c r="N3">
-        <v>40.49436870247035</v>
-      </c>
-      <c r="O3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -622,13 +619,13 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>148900</v>
+        <v>149300</v>
       </c>
       <c r="E4">
-        <v>92</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F4">
-        <v>7.12</v>
+        <v>7.56</v>
       </c>
       <c r="G4">
         <v>50</v>
@@ -637,25 +634,25 @@
         <v>63</v>
       </c>
       <c r="I4">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="J4">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4">
-        <v>49.5</v>
+        <v>53.5</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4">
+        <v>40.44495449250464</v>
+      </c>
+      <c r="O4" t="s">
         <v>30</v>
-      </c>
-      <c r="N4">
-        <v>40.49436870247035</v>
-      </c>
-      <c r="O4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -669,40 +666,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>85200</v>
+        <v>85700</v>
       </c>
       <c r="E5">
-        <v>81.5</v>
+        <v>85.7</v>
       </c>
       <c r="F5">
-        <v>18.5</v>
+        <v>15.81</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I5">
         <v>60</v>
       </c>
       <c r="J5">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="K5">
-        <v>48.1</v>
+        <v>51.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5">
+        <v>40.44495449250464</v>
+      </c>
+      <c r="O5" t="s">
         <v>30</v>
-      </c>
-      <c r="N5">
-        <v>40.49436870247035</v>
-      </c>
-      <c r="O5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -743,13 +740,13 @@
         <v>28</v>
       </c>
       <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6">
+        <v>40.44495449250464</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
-      </c>
-      <c r="N6">
-        <v>40.49436870247035</v>
-      </c>
-      <c r="O6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -790,13 +787,13 @@
         <v>28</v>
       </c>
       <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7">
+        <v>40.44495449250464</v>
+      </c>
+      <c r="O7" t="s">
         <v>30</v>
-      </c>
-      <c r="N7">
-        <v>40.49436870247035</v>
-      </c>
-      <c r="O7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-03-03 23:00:08
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -61,52 +61,55 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-01-19</t>
+    <t>2026-03-03</t>
+  </si>
+  <si>
+    <t>SamsungElec</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
+  </si>
+  <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
-    <t>SamsungElec</t>
+    <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
     <t>DB HiTek</t>
   </si>
   <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
+    <t>005930.KS</t>
   </si>
   <si>
     <t>000660.KS</t>
   </si>
   <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
     <t>240810.KS</t>
   </si>
   <si>
-    <t>005930.KS</t>
+    <t>403870.KS</t>
   </si>
   <si>
     <t>000990.KS</t>
   </si>
   <si>
-    <t>058470.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
   </si>
   <si>
-    <t>⚪ 중립 구간</t>
+    <t>🤏 바닥권 접근 구간입니다.</t>
+  </si>
+  <si>
+    <t>🔴 강한 긴축 / 리스크</t>
   </si>
 </sst>
 </file>
@@ -525,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>764000</v>
+        <v>195100</v>
       </c>
       <c r="E2">
-        <v>89.09999999999999</v>
+        <v>71.3</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1.09</v>
       </c>
       <c r="G2">
         <v>50</v>
       </c>
       <c r="H2">
+        <v>73</v>
+      </c>
+      <c r="I2">
         <v>80</v>
       </c>
-      <c r="I2">
-        <v>76</v>
-      </c>
       <c r="J2">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="K2">
-        <v>57.5</v>
+        <v>53.1</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -572,28 +575,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>76700</v>
+        <v>939000</v>
       </c>
       <c r="E3">
-        <v>67.3</v>
+        <v>60</v>
       </c>
       <c r="F3">
-        <v>2.27</v>
+        <v>-1.08</v>
       </c>
       <c r="G3">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H3">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I3">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J3">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="K3">
-        <v>56.5</v>
+        <v>50.3</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,10 +605,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,28 +622,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>149300</v>
+        <v>106200</v>
       </c>
       <c r="E4">
-        <v>90.90000000000001</v>
+        <v>63</v>
       </c>
       <c r="F4">
-        <v>7.56</v>
+        <v>10.05</v>
       </c>
       <c r="G4">
         <v>50</v>
       </c>
       <c r="H4">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="J4">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="K4">
-        <v>53.5</v>
+        <v>42.3</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,10 +652,10 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -666,28 +669,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>85700</v>
+        <v>125600</v>
       </c>
       <c r="E5">
-        <v>85.7</v>
+        <v>56.2</v>
       </c>
       <c r="F5">
-        <v>15.81</v>
+        <v>5.28</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="H5">
+        <v>50</v>
+      </c>
+      <c r="I5">
         <v>53</v>
       </c>
-      <c r="I5">
-        <v>60</v>
-      </c>
       <c r="J5">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="K5">
-        <v>51.1</v>
+        <v>42.3</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,10 +699,10 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -713,28 +716,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>64700</v>
+        <v>44850</v>
       </c>
       <c r="E6">
-        <v>64.59999999999999</v>
+        <v>47.4</v>
       </c>
       <c r="F6">
-        <v>3.19</v>
+        <v>-2.29</v>
       </c>
       <c r="G6">
+        <v>30</v>
+      </c>
+      <c r="H6">
+        <v>53</v>
+      </c>
+      <c r="I6">
+        <v>53</v>
+      </c>
+      <c r="J6">
         <v>60</v>
       </c>
-      <c r="H6">
-        <v>56</v>
-      </c>
-      <c r="I6">
-        <v>43</v>
-      </c>
-      <c r="J6">
-        <v>66</v>
-      </c>
       <c r="K6">
-        <v>47.3</v>
+        <v>36.3</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,10 +746,10 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,40 +763,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>35750</v>
+        <v>90500</v>
       </c>
       <c r="E7">
-        <v>63.9</v>
+        <v>25.8</v>
       </c>
       <c r="F7">
-        <v>8.01</v>
+        <v>-2.69</v>
       </c>
       <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>56</v>
+      </c>
+      <c r="I7">
         <v>60</v>
       </c>
-      <c r="H7">
-        <v>36</v>
-      </c>
-      <c r="I7">
-        <v>36</v>
-      </c>
       <c r="J7">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="K7">
-        <v>44.5</v>
+        <v>33.1</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7">
-        <v>40.44495449250464</v>
+        <v>20.49503599836755</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-03-09 09:23:23
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>날짜</t>
   </si>
@@ -61,21 +61,21 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-03-03</t>
+    <t>2026-03-09</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>SK hynix</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
@@ -85,15 +85,15 @@
     <t>005930.KS</t>
   </si>
   <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>000660.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
   </si>
   <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
     <t>403870.KS</t>
   </si>
   <si>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
-  </si>
-  <si>
-    <t>🤏 바닥권 접근 구간입니다.</t>
   </si>
   <si>
     <t>🔴 강한 긴축 / 리스크</t>
@@ -528,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>195100</v>
+        <v>173100</v>
       </c>
       <c r="E2">
-        <v>71.3</v>
+        <v>52</v>
       </c>
       <c r="F2">
-        <v>1.09</v>
+        <v>-20.05</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H2">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K2">
-        <v>53.1</v>
+        <v>43.5</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,10 +555,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>20.49503599836755</v>
+        <v>4.469434098808478</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -575,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>939000</v>
+        <v>137800</v>
       </c>
       <c r="E3">
-        <v>60</v>
+        <v>62.2</v>
       </c>
       <c r="F3">
-        <v>-1.08</v>
+        <v>8.93</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I3">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="J3">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K3">
-        <v>50.3</v>
+        <v>41.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,10 +602,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>20.49503599836755</v>
+        <v>4.469434098808478</v>
       </c>
       <c r="O3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -622,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>106200</v>
+        <v>852000</v>
       </c>
       <c r="E4">
-        <v>63</v>
+        <v>49.5</v>
       </c>
       <c r="F4">
-        <v>10.05</v>
+        <v>-19.7</v>
       </c>
       <c r="G4">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H4">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="I4">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="J4">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K4">
-        <v>42.3</v>
+        <v>40.5</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -652,10 +649,10 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>20.49503599836755</v>
+        <v>4.469434098808478</v>
       </c>
       <c r="O4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -669,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>125600</v>
+        <v>127000</v>
       </c>
       <c r="E5">
-        <v>56.2</v>
+        <v>73.5</v>
       </c>
       <c r="F5">
-        <v>5.28</v>
+        <v>18.91</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="I5">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="J5">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="K5">
-        <v>42.3</v>
+        <v>38.5</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,10 +696,10 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>20.49503599836755</v>
+        <v>4.469434098808478</v>
       </c>
       <c r="O5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -716,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>44850</v>
+        <v>47850</v>
       </c>
       <c r="E6">
-        <v>47.4</v>
+        <v>55.6</v>
       </c>
       <c r="F6">
-        <v>-2.29</v>
+        <v>10.51</v>
       </c>
       <c r="G6">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I6">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="K6">
-        <v>36.3</v>
+        <v>38.5</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -746,10 +743,10 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>20.49503599836755</v>
+        <v>4.469434098808478</v>
       </c>
       <c r="O6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -763,40 +760,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>90500</v>
+        <v>83600</v>
       </c>
       <c r="E7">
-        <v>25.8</v>
+        <v>42.1</v>
       </c>
       <c r="F7">
-        <v>-2.69</v>
+        <v>-11.85</v>
       </c>
       <c r="G7">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H7">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I7">
         <v>60</v>
       </c>
       <c r="J7">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K7">
-        <v>33.1</v>
+        <v>31.3</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7">
+        <v>4.469434098808478</v>
+      </c>
+      <c r="O7" t="s">
         <v>30</v>
-      </c>
-      <c r="N7">
-        <v>20.49503599836755</v>
-      </c>
-      <c r="O7" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-03-09 17:05:30
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>⛔ 관망하십시오.</t>
+  </si>
+  <si>
+    <t>🤏 바닥권 접근 구간입니다.</t>
   </si>
   <si>
     <t>🔴 강한 긴축 / 리스크</t>
@@ -525,13 +528,13 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>173100</v>
+        <v>173500</v>
       </c>
       <c r="E2">
-        <v>52</v>
+        <v>52.1</v>
       </c>
       <c r="F2">
-        <v>-20.05</v>
+        <v>-19.86</v>
       </c>
       <c r="G2">
         <v>30</v>
@@ -546,7 +549,7 @@
         <v>83</v>
       </c>
       <c r="K2">
-        <v>43.5</v>
+        <v>42.2</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -593,7 +596,7 @@
         <v>86</v>
       </c>
       <c r="K3">
-        <v>41.5</v>
+        <v>40.2</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,10 +605,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,13 +622,13 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>852000</v>
+        <v>836000</v>
       </c>
       <c r="E4">
-        <v>49.5</v>
+        <v>48.4</v>
       </c>
       <c r="F4">
-        <v>-19.7</v>
+        <v>-21.21</v>
       </c>
       <c r="G4">
         <v>20</v>
@@ -640,19 +643,19 @@
         <v>80</v>
       </c>
       <c r="K4">
-        <v>40.5</v>
+        <v>39.2</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -687,7 +690,7 @@
         <v>66</v>
       </c>
       <c r="K5">
-        <v>38.5</v>
+        <v>37.2</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,10 +699,10 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -734,7 +737,7 @@
         <v>66</v>
       </c>
       <c r="K6">
-        <v>38.5</v>
+        <v>37.2</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,10 +746,10 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,13 +763,13 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>83600</v>
+        <v>83200</v>
       </c>
       <c r="E7">
-        <v>42.1</v>
+        <v>41.8</v>
       </c>
       <c r="F7">
-        <v>-11.85</v>
+        <v>-12.27</v>
       </c>
       <c r="G7">
         <v>20</v>
@@ -781,7 +784,7 @@
         <v>63</v>
       </c>
       <c r="K7">
-        <v>31.3</v>
+        <v>30</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,10 +793,10 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>4.469434098808478</v>
+        <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-03-10 13:32:58
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,7 +61,10 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-03-09</t>
+    <t>2026-03-10</t>
+  </si>
+  <si>
+    <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
     <t>SamsungElec</t>
@@ -73,15 +76,15 @@
     <t>SK hynix</t>
   </si>
   <si>
-    <t>058470.KS,0P0000ASU1,98886</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
     <t>DB HiTek</t>
   </si>
   <si>
+    <t>058470.KS</t>
+  </si>
+  <si>
     <t>005930.KS</t>
   </si>
   <si>
@@ -91,9 +94,6 @@
     <t>000660.KS</t>
   </si>
   <si>
-    <t>058470.KS</t>
-  </si>
-  <si>
     <t>403870.KS</t>
   </si>
   <si>
@@ -109,7 +109,7 @@
     <t>🤏 바닥권 접근 구간입니다.</t>
   </si>
   <si>
-    <t>🔴 강한 긴축 / 리스크</t>
+    <t>🟠 하락 우위 (긴장 구간)</t>
   </si>
 </sst>
 </file>
@@ -528,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>173500</v>
+        <v>118200</v>
       </c>
       <c r="E2">
-        <v>52.1</v>
+        <v>66.2</v>
       </c>
       <c r="F2">
-        <v>-19.86</v>
+        <v>11.3</v>
       </c>
       <c r="G2">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H2">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="I2">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="J2">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="K2">
-        <v>42.2</v>
+        <v>54.1</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,28 +575,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>137800</v>
+        <v>186100</v>
       </c>
       <c r="E3">
-        <v>62.2</v>
+        <v>52.8</v>
       </c>
       <c r="F3">
-        <v>8.93</v>
+        <v>-4.61</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="H3">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="I3">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="J3">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K3">
-        <v>40.2</v>
+        <v>50.7</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,7 +605,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -622,37 +622,37 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>836000</v>
+        <v>124300</v>
       </c>
       <c r="E4">
-        <v>48.4</v>
+        <v>57.2</v>
       </c>
       <c r="F4">
-        <v>-21.21</v>
+        <v>-1.04</v>
       </c>
       <c r="G4">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I4">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="J4">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="K4">
-        <v>39.2</v>
+        <v>48.1</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -669,28 +669,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>127000</v>
+        <v>919000</v>
       </c>
       <c r="E5">
-        <v>73.5</v>
+        <v>52.2</v>
       </c>
       <c r="F5">
-        <v>18.91</v>
+        <v>-2.13</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H5">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="I5">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="J5">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="K5">
-        <v>37.2</v>
+        <v>46.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -716,37 +716,37 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>47850</v>
+        <v>43500</v>
       </c>
       <c r="E6">
-        <v>55.6</v>
+        <v>50.4</v>
       </c>
       <c r="F6">
-        <v>10.51</v>
+        <v>-3.01</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H6">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I6">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="J6">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="K6">
-        <v>37.2</v>
+        <v>39.7</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,13 +763,13 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>83200</v>
+        <v>86200</v>
       </c>
       <c r="E7">
-        <v>41.8</v>
+        <v>43.7</v>
       </c>
       <c r="F7">
-        <v>-12.27</v>
+        <v>-3.89</v>
       </c>
       <c r="G7">
         <v>20</v>
@@ -778,13 +778,13 @@
         <v>50</v>
       </c>
       <c r="I7">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="J7">
         <v>63</v>
       </c>
       <c r="K7">
-        <v>30</v>
+        <v>38.1</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -793,7 +793,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>32.23518188264562</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Auto update: 2026-03-10 15:44:27
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -67,15 +67,15 @@
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
+    <t>SK hynix</t>
+  </si>
+  <si>
     <t>SamsungElec</t>
   </si>
   <si>
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
-    <t>SK hynix</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
@@ -85,13 +85,13 @@
     <t>058470.KS</t>
   </si>
   <si>
+    <t>000660.KS</t>
+  </si>
+  <si>
     <t>005930.KS</t>
   </si>
   <si>
     <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000660.KS</t>
   </si>
   <si>
     <t>403870.KS</t>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,19 +575,19 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>186100</v>
+        <v>943000</v>
       </c>
       <c r="E3">
-        <v>52.8</v>
+        <v>53.6</v>
       </c>
       <c r="F3">
-        <v>-4.61</v>
+        <v>0.43</v>
       </c>
       <c r="G3">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I3">
         <v>80</v>
@@ -596,7 +596,7 @@
         <v>80</v>
       </c>
       <c r="K3">
-        <v>50.7</v>
+        <v>53.7</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,7 +605,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -622,28 +622,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>124300</v>
+        <v>187900</v>
       </c>
       <c r="E4">
-        <v>57.2</v>
+        <v>53.4</v>
       </c>
       <c r="F4">
-        <v>-1.04</v>
+        <v>-3.69</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I4">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="J4">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="K4">
-        <v>48.1</v>
+        <v>50.7</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -652,7 +652,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -669,28 +669,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>919000</v>
+        <v>124300</v>
       </c>
       <c r="E5">
-        <v>52.2</v>
+        <v>57.2</v>
       </c>
       <c r="F5">
-        <v>-2.13</v>
+        <v>-1.04</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I5">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="J5">
         <v>76</v>
       </c>
       <c r="K5">
-        <v>46.1</v>
+        <v>48.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
       <c r="N6">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,19 +763,19 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>86200</v>
+        <v>87800</v>
       </c>
       <c r="E7">
-        <v>43.7</v>
+        <v>45.1</v>
       </c>
       <c r="F7">
-        <v>-3.89</v>
+        <v>-2.1</v>
       </c>
       <c r="G7">
         <v>20</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I7">
         <v>56</v>
@@ -793,7 +793,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>32.23518188264562</v>
+        <v>32.42054265786911</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Auto update: 2026-03-11 12:27:33
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>날짜</t>
   </si>
@@ -61,21 +61,21 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-03-10</t>
+    <t>2026-03-11</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
     <t>SK hynix</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
@@ -85,15 +85,15 @@
     <t>058470.KS</t>
   </si>
   <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
     <t>000660.KS</t>
   </si>
   <si>
     <t>005930.KS</t>
   </si>
   <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
     <t>403870.KS</t>
   </si>
   <si>
@@ -106,10 +106,7 @@
     <t>⛔ 관망하십시오.</t>
   </si>
   <si>
-    <t>🤏 바닥권 접근 구간입니다.</t>
-  </si>
-  <si>
-    <t>🟠 하락 우위 (긴장 구간)</t>
+    <t>⚪ 중립 구간</t>
   </si>
 </sst>
 </file>
@@ -528,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>118200</v>
+        <v>119500</v>
       </c>
       <c r="E2">
-        <v>66.2</v>
+        <v>65.3</v>
       </c>
       <c r="F2">
-        <v>11.3</v>
+        <v>7.17</v>
       </c>
       <c r="G2">
         <v>60</v>
       </c>
       <c r="H2">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="I2">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J2">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="K2">
-        <v>54.1</v>
+        <v>59</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,10 +555,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>32.42054265786911</v>
+        <v>43.44936356612781</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -575,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>943000</v>
+        <v>125900</v>
       </c>
       <c r="E3">
-        <v>53.6</v>
+        <v>46.9</v>
       </c>
       <c r="F3">
-        <v>0.43</v>
+        <v>1.94</v>
       </c>
       <c r="G3">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H3">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I3">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J3">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="K3">
-        <v>53.7</v>
+        <v>57.2</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -605,10 +602,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>32.42054265786911</v>
+        <v>43.44936356612781</v>
       </c>
       <c r="O3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -622,16 +619,16 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>187900</v>
+        <v>979000</v>
       </c>
       <c r="E4">
-        <v>53.4</v>
+        <v>56.2</v>
       </c>
       <c r="F4">
-        <v>-3.69</v>
+        <v>15.31</v>
       </c>
       <c r="G4">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H4">
         <v>80</v>
@@ -640,10 +637,10 @@
         <v>80</v>
       </c>
       <c r="J4">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="K4">
-        <v>50.7</v>
+        <v>57</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -652,10 +649,10 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>32.42054265786911</v>
+        <v>43.44936356612781</v>
       </c>
       <c r="O4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -669,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>124300</v>
+        <v>192800</v>
       </c>
       <c r="E5">
-        <v>57.2</v>
+        <v>54.2</v>
       </c>
       <c r="F5">
-        <v>-1.04</v>
+        <v>11.96</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="I5">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J5">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="K5">
-        <v>48.1</v>
+        <v>53.2</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,10 +696,10 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>32.42054265786911</v>
+        <v>43.44936356612781</v>
       </c>
       <c r="O5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -716,40 +713,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>43500</v>
+        <v>45700</v>
       </c>
       <c r="E6">
-        <v>50.4</v>
+        <v>54.4</v>
       </c>
       <c r="F6">
-        <v>-3.01</v>
+        <v>5.79</v>
       </c>
       <c r="G6">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="J6">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K6">
-        <v>39.7</v>
+        <v>47.4</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6">
+        <v>43.44936356612781</v>
+      </c>
+      <c r="O6" t="s">
         <v>30</v>
-      </c>
-      <c r="N6">
-        <v>32.42054265786911</v>
-      </c>
-      <c r="O6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -763,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>87800</v>
+        <v>87200</v>
       </c>
       <c r="E7">
-        <v>45.1</v>
+        <v>46</v>
       </c>
       <c r="F7">
-        <v>-2.1</v>
+        <v>13.83</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H7">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I7">
         <v>56</v>
       </c>
       <c r="J7">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K7">
-        <v>38.1</v>
+        <v>44.4</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -793,10 +790,10 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>32.42054265786911</v>
+        <v>43.44936356612781</v>
       </c>
       <c r="O7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-03-12 18:59:45
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,7 +61,7 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-03-11</t>
+    <t>2026-03-12</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
@@ -70,15 +70,15 @@
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
     <t>SK hynix</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
-  </si>
-  <si>
     <t>DB HiTek</t>
   </si>
   <si>
@@ -88,13 +88,13 @@
     <t>240810.KS</t>
   </si>
   <si>
+    <t>403870.KS</t>
+  </si>
+  <si>
     <t>000660.KS</t>
   </si>
   <si>
     <t>005930.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
   </si>
   <si>
     <t>000990.KS</t>
@@ -525,28 +525,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>119500</v>
+        <v>113700</v>
       </c>
       <c r="E2">
-        <v>65.3</v>
+        <v>60.8</v>
       </c>
       <c r="F2">
-        <v>7.17</v>
+        <v>12.69</v>
       </c>
       <c r="G2">
         <v>60</v>
       </c>
       <c r="H2">
+        <v>63</v>
+      </c>
+      <c r="I2">
+        <v>66</v>
+      </c>
+      <c r="J2">
         <v>70</v>
       </c>
-      <c r="I2">
-        <v>70</v>
-      </c>
-      <c r="J2">
-        <v>83</v>
-      </c>
       <c r="K2">
-        <v>59</v>
+        <v>56.9</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -572,28 +572,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>125900</v>
+        <v>120000</v>
       </c>
       <c r="E3">
-        <v>46.9</v>
+        <v>55.3</v>
       </c>
       <c r="F3">
-        <v>1.94</v>
+        <v>11.63</v>
       </c>
       <c r="G3">
         <v>50</v>
       </c>
       <c r="H3">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="I3">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J3">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="K3">
-        <v>57.2</v>
+        <v>55.5</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -619,28 +619,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>979000</v>
+        <v>43600</v>
       </c>
       <c r="E4">
-        <v>56.2</v>
+        <v>51.3</v>
       </c>
       <c r="F4">
-        <v>15.31</v>
+        <v>14.89</v>
       </c>
       <c r="G4">
         <v>40</v>
       </c>
       <c r="H4">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="I4">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="J4">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="K4">
-        <v>57</v>
+        <v>49.7</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -666,28 +666,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>192800</v>
+        <v>930000</v>
       </c>
       <c r="E5">
-        <v>54.2</v>
+        <v>52.4</v>
       </c>
       <c r="F5">
-        <v>11.96</v>
+        <v>-1.17</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H5">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I5">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="J5">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="K5">
-        <v>53.2</v>
+        <v>46.5</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -713,28 +713,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>45700</v>
+        <v>187900</v>
       </c>
       <c r="E6">
-        <v>54.4</v>
+        <v>49.2</v>
       </c>
       <c r="F6">
-        <v>5.79</v>
+        <v>-1.93</v>
       </c>
       <c r="G6">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H6">
+        <v>66</v>
+      </c>
+      <c r="I6">
         <v>60</v>
       </c>
-      <c r="I6">
-        <v>56</v>
-      </c>
       <c r="J6">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="K6">
-        <v>47.4</v>
+        <v>45.5</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -760,28 +760,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>87200</v>
+        <v>85900</v>
       </c>
       <c r="E7">
-        <v>46</v>
+        <v>46.3</v>
       </c>
       <c r="F7">
-        <v>13.83</v>
+        <v>-8.76</v>
       </c>
       <c r="G7">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H7">
         <v>46</v>
       </c>
       <c r="I7">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J7">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K7">
-        <v>44.4</v>
+        <v>39.7</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>43.44936356612781</v>
+        <v>41.74287521812095</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-03-12 19:02:55
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -555,7 +555,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O2" t="s">
         <v>30</v>
@@ -602,7 +602,7 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O3" t="s">
         <v>30</v>
@@ -649,7 +649,7 @@
         <v>29</v>
       </c>
       <c r="N4">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -696,7 +696,7 @@
         <v>29</v>
       </c>
       <c r="N5">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -743,7 +743,7 @@
         <v>29</v>
       </c>
       <c r="N6">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -790,7 +790,7 @@
         <v>29</v>
       </c>
       <c r="N7">
-        <v>41.74287521812095</v>
+        <v>41.81508460778518</v>
       </c>
       <c r="O7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Auto update: 2026-04-08 12:32:42
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -61,7 +61,13 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-03-12</t>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>SamsungElec</t>
+  </si>
+  <si>
+    <t>SK hynix</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
@@ -70,16 +76,16 @@
     <t>240810.KS,0P00017YB3,330568</t>
   </si>
   <si>
+    <t>DB HiTek</t>
+  </si>
+  <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>SK hynix</t>
-  </si>
-  <si>
-    <t>SamsungElec</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
+    <t>005930.KS</t>
+  </si>
+  <si>
+    <t>000660.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
@@ -88,25 +94,22 @@
     <t>240810.KS</t>
   </si>
   <si>
+    <t>000990.KS</t>
+  </si>
+  <si>
     <t>403870.KS</t>
   </si>
   <si>
-    <t>000660.KS</t>
-  </si>
-  <si>
-    <t>005930.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
   </si>
   <si>
+    <t>📈 매수 관찰 구간입니다.</t>
+  </si>
+  <si>
     <t>⛔ 관망하십시오.</t>
   </si>
   <si>
-    <t>⚪ 중립 구간</t>
+    <t>🟢 상승 우위 (다소 완화)</t>
   </si>
 </sst>
 </file>
@@ -525,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>113700</v>
+        <v>210500</v>
       </c>
       <c r="E2">
-        <v>60.8</v>
+        <v>54.7</v>
       </c>
       <c r="F2">
-        <v>12.69</v>
+        <v>10.99</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H2">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I2">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J2">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="K2">
-        <v>56.9</v>
+        <v>64.2</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -555,10 +558,10 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -572,28 +575,28 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>120000</v>
+        <v>1008000</v>
       </c>
       <c r="E3">
-        <v>55.3</v>
+        <v>49.6</v>
       </c>
       <c r="F3">
-        <v>11.63</v>
+        <v>12.37</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I3">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J3">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="K3">
-        <v>55.5</v>
+        <v>61.2</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
@@ -602,10 +605,10 @@
         <v>29</v>
       </c>
       <c r="N3">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -619,40 +622,40 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>43600</v>
+        <v>109700</v>
       </c>
       <c r="E4">
-        <v>51.3</v>
+        <v>44.3</v>
       </c>
       <c r="F4">
-        <v>14.89</v>
+        <v>16.21</v>
       </c>
       <c r="G4">
         <v>40</v>
       </c>
       <c r="H4">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="I4">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="J4">
+        <v>73</v>
+      </c>
+      <c r="K4">
         <v>60</v>
-      </c>
-      <c r="K4">
-        <v>49.7</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -666,40 +669,40 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>930000</v>
+        <v>114100</v>
       </c>
       <c r="E5">
-        <v>52.4</v>
+        <v>43.9</v>
       </c>
       <c r="F5">
-        <v>-1.17</v>
+        <v>5.55</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H5">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I5">
         <v>70</v>
       </c>
       <c r="J5">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="K5">
-        <v>46.5</v>
+        <v>57</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N5">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -713,40 +716,40 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>187900</v>
+        <v>92100</v>
       </c>
       <c r="E6">
-        <v>49.2</v>
+        <v>55</v>
       </c>
       <c r="F6">
-        <v>-1.93</v>
+        <v>7.09</v>
       </c>
       <c r="G6">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H6">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="J6">
-        <v>80</v>
+        <v>46</v>
       </c>
       <c r="K6">
-        <v>45.5</v>
+        <v>54</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N6">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -760,40 +763,40 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>85900</v>
+        <v>41650</v>
       </c>
       <c r="E7">
-        <v>46.3</v>
+        <v>32.1</v>
       </c>
       <c r="F7">
-        <v>-8.76</v>
+        <v>1.83</v>
       </c>
       <c r="G7">
         <v>20</v>
       </c>
       <c r="H7">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="I7">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="J7">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K7">
-        <v>39.7</v>
+        <v>42</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7">
-        <v>41.81508460778518</v>
+        <v>66.57973643566133</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: 2026-05-07 15:04:55
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,45 +61,45 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-04-08</t>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>SK hynix</t>
   </si>
   <si>
     <t>SamsungElec</t>
   </si>
   <si>
-    <t>SK hynix</t>
+    <t>403870.KS,0P0001PE9K,566428</t>
+  </si>
+  <si>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
+    <t>DB HiTek</t>
   </si>
   <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
-    <t>403870.KS,0P0001PE9K,566428</t>
+    <t>000660.KS</t>
   </si>
   <si>
     <t>005930.KS</t>
   </si>
   <si>
-    <t>000660.KS</t>
+    <t>403870.KS</t>
+  </si>
+  <si>
+    <t>240810.KS</t>
+  </si>
+  <si>
+    <t>000990.KS</t>
   </si>
   <si>
     <t>058470.KS</t>
   </si>
   <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
-    <t>403870.KS</t>
-  </si>
-  <si>
     <t>Pattern</t>
   </si>
   <si>
@@ -109,7 +109,7 @@
     <t>⛔ 관망하십시오.</t>
   </si>
   <si>
-    <t>🟢 상승 우위 (다소 완화)</t>
+    <t>⚪ 중립 구간</t>
   </si>
 </sst>
 </file>
@@ -528,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>210500</v>
+        <v>1662000</v>
       </c>
       <c r="E2">
-        <v>54.7</v>
+        <v>92.7</v>
       </c>
       <c r="F2">
-        <v>10.99</v>
+        <v>27.85</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I2">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="J2">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K2">
-        <v>64.2</v>
+        <v>61.7</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,37 +575,37 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>1008000</v>
+        <v>272500</v>
       </c>
       <c r="E3">
-        <v>49.6</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="F3">
-        <v>12.37</v>
+        <v>22.75</v>
       </c>
       <c r="G3">
         <v>40</v>
       </c>
       <c r="H3">
+        <v>66</v>
+      </c>
+      <c r="I3">
         <v>70</v>
       </c>
-      <c r="I3">
-        <v>73</v>
-      </c>
       <c r="J3">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="K3">
-        <v>61.2</v>
+        <v>57.7</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -622,28 +622,28 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>109700</v>
+        <v>56600</v>
       </c>
       <c r="E4">
-        <v>44.3</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="F4">
-        <v>16.21</v>
+        <v>3.28</v>
       </c>
       <c r="G4">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H4">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I4">
+        <v>60</v>
+      </c>
+      <c r="J4">
         <v>70</v>
       </c>
-      <c r="J4">
-        <v>73</v>
-      </c>
       <c r="K4">
-        <v>60</v>
+        <v>56.7</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
@@ -652,7 +652,7 @@
         <v>30</v>
       </c>
       <c r="N4">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -669,28 +669,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>114100</v>
+        <v>129000</v>
       </c>
       <c r="E5">
-        <v>43.9</v>
+        <v>58.6</v>
       </c>
       <c r="F5">
-        <v>5.55</v>
+        <v>6.17</v>
       </c>
       <c r="G5">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H5">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I5">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="J5">
         <v>86</v>
       </c>
       <c r="K5">
-        <v>57</v>
+        <v>55.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>30</v>
       </c>
       <c r="N5">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -716,28 +716,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>92100</v>
+        <v>155800</v>
       </c>
       <c r="E6">
-        <v>55</v>
+        <v>81.2</v>
       </c>
       <c r="F6">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="G6">
+        <v>50</v>
+      </c>
+      <c r="H6">
+        <v>46</v>
+      </c>
+      <c r="I6">
+        <v>53</v>
+      </c>
+      <c r="J6">
         <v>60</v>
       </c>
-      <c r="H6">
-        <v>53</v>
-      </c>
-      <c r="I6">
-        <v>40</v>
-      </c>
-      <c r="J6">
-        <v>46</v>
-      </c>
       <c r="K6">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
       <c r="N6">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,28 +763,28 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>41650</v>
+        <v>116700</v>
       </c>
       <c r="E7">
-        <v>32.1</v>
+        <v>56</v>
       </c>
       <c r="F7">
-        <v>1.83</v>
+        <v>6.28</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="I7">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="J7">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="K7">
-        <v>42</v>
+        <v>51.1</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
@@ -793,7 +793,7 @@
         <v>30</v>
       </c>
       <c r="N7">
-        <v>66.57973643566133</v>
+        <v>59.14876667115259</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Auto update: 2026-06-07 01:21:22
</commit_message>
<xml_diff>
--- a/DECISION/국장_반도체_분석.xlsx
+++ b/DECISION/국장_반도체_분석.xlsx
@@ -61,55 +61,55 @@
     <t>MACRO_SIGNAL</t>
   </si>
   <si>
-    <t>2026-05-07</t>
+    <t>2026-06-07</t>
+  </si>
+  <si>
+    <t>SamsungElec</t>
   </si>
   <si>
     <t>SK hynix</t>
   </si>
   <si>
-    <t>SamsungElec</t>
+    <t>240810.KS,0P00017YB3,330568</t>
+  </si>
+  <si>
+    <t>DB HiTek</t>
   </si>
   <si>
     <t>403870.KS,0P0001PE9K,566428</t>
   </si>
   <si>
-    <t>240810.KS,0P00017YB3,330568</t>
-  </si>
-  <si>
-    <t>DB HiTek</t>
-  </si>
-  <si>
     <t>058470.KS,0P0000ASU1,98886</t>
   </si>
   <si>
+    <t>005930.KS</t>
+  </si>
+  <si>
     <t>000660.KS</t>
   </si>
   <si>
-    <t>005930.KS</t>
+    <t>240810.KS</t>
+  </si>
+  <si>
+    <t>000990.KS</t>
   </si>
   <si>
     <t>403870.KS</t>
   </si>
   <si>
-    <t>240810.KS</t>
-  </si>
-  <si>
-    <t>000990.KS</t>
-  </si>
-  <si>
     <t>058470.KS</t>
   </si>
   <si>
     <t>Pattern</t>
   </si>
   <si>
-    <t>📈 매수 관찰 구간입니다.</t>
-  </si>
-  <si>
     <t>⛔ 관망하십시오.</t>
   </si>
   <si>
-    <t>⚪ 중립 구간</t>
+    <t>🤏 바닥권 접근 구간입니다.</t>
+  </si>
+  <si>
+    <t>🔴 강한 긴축 / 리스크</t>
   </si>
 </sst>
 </file>
@@ -528,28 +528,28 @@
         <v>22</v>
       </c>
       <c r="D2">
-        <v>1662000</v>
+        <v>329000</v>
       </c>
       <c r="E2">
-        <v>92.7</v>
+        <v>58.8</v>
       </c>
       <c r="F2">
-        <v>27.85</v>
+        <v>9.85</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H2">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I2">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="J2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K2">
-        <v>61.7</v>
+        <v>56.3</v>
       </c>
       <c r="L2" t="s">
         <v>28</v>
@@ -558,7 +558,7 @@
         <v>29</v>
       </c>
       <c r="N2">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O2" t="s">
         <v>31</v>
@@ -575,37 +575,37 @@
         <v>23</v>
       </c>
       <c r="D3">
-        <v>272500</v>
+        <v>2070000</v>
       </c>
       <c r="E3">
-        <v>81.90000000000001</v>
+        <v>54.3</v>
       </c>
       <c r="F3">
-        <v>22.75</v>
+        <v>-9.57</v>
       </c>
       <c r="G3">
         <v>40</v>
       </c>
       <c r="H3">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I3">
         <v>70</v>
       </c>
       <c r="J3">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="K3">
-        <v>57.7</v>
+        <v>43.9</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N3">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O3" t="s">
         <v>31</v>
@@ -622,37 +622,37 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>56600</v>
+        <v>132700</v>
       </c>
       <c r="E4">
-        <v>87.59999999999999</v>
+        <v>52.8</v>
       </c>
       <c r="F4">
-        <v>3.28</v>
+        <v>22.53</v>
       </c>
       <c r="G4">
         <v>50</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="I4">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J4">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="K4">
-        <v>56.7</v>
+        <v>36.1</v>
       </c>
       <c r="L4" t="s">
         <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N4">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O4" t="s">
         <v>31</v>
@@ -669,28 +669,28 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <v>129000</v>
+        <v>173800</v>
       </c>
       <c r="E5">
-        <v>58.6</v>
+        <v>47.2</v>
       </c>
       <c r="F5">
-        <v>6.17</v>
+        <v>-10.55</v>
       </c>
       <c r="G5">
+        <v>20</v>
+      </c>
+      <c r="H5">
         <v>50</v>
       </c>
-      <c r="H5">
-        <v>56</v>
-      </c>
       <c r="I5">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J5">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="K5">
-        <v>55.1</v>
+        <v>35.1</v>
       </c>
       <c r="L5" t="s">
         <v>28</v>
@@ -699,7 +699,7 @@
         <v>30</v>
       </c>
       <c r="N5">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O5" t="s">
         <v>31</v>
@@ -716,28 +716,28 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>155800</v>
+        <v>50300</v>
       </c>
       <c r="E6">
-        <v>81.2</v>
+        <v>45.2</v>
       </c>
       <c r="F6">
-        <v>0.71</v>
+        <v>-1.18</v>
       </c>
       <c r="G6">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H6">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I6">
         <v>53</v>
       </c>
       <c r="J6">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="K6">
-        <v>53.9</v>
+        <v>31.1</v>
       </c>
       <c r="L6" t="s">
         <v>28</v>
@@ -746,7 +746,7 @@
         <v>30</v>
       </c>
       <c r="N6">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O6" t="s">
         <v>31</v>
@@ -763,37 +763,37 @@
         <v>27</v>
       </c>
       <c r="D7">
-        <v>116700</v>
+        <v>94100</v>
       </c>
       <c r="E7">
+        <v>34.1</v>
+      </c>
+      <c r="F7">
+        <v>-5.05</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>46</v>
+      </c>
+      <c r="I7">
         <v>56</v>
       </c>
-      <c r="F7">
-        <v>6.28</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>63</v>
-      </c>
-      <c r="I7">
-        <v>46</v>
-      </c>
       <c r="J7">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K7">
-        <v>51.1</v>
+        <v>29.3</v>
       </c>
       <c r="L7" t="s">
         <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N7">
-        <v>59.14876667115259</v>
+        <v>13.11002090356014</v>
       </c>
       <c r="O7" t="s">
         <v>31</v>

</xml_diff>